<commit_message>
added more possible coproducts in template excel
</commit_message>
<xml_diff>
--- a/01_create_system_expansion/templates/reaction_extension_layer.xlsx
+++ b/01_create_system_expansion/templates/reaction_extension_layer.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\gossen\Projects\cm-py\DatabaseGeneration-02_techModel\01_create_system_expansion\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\gossen\Projects\DB_Improvement\DatabaseGeneration-02_techModel\01_create_system_expansion\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A695D89-6818-4358-8FD4-D6B5CB5B96AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D40AC47E-E838-45DC-B860-DA024CF25A91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4425" yWindow="3810" windowWidth="21600" windowHeight="11295" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-4965" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="matrix_table" sheetId="9" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="37">
   <si>
     <t>raw_material_id</t>
   </si>
@@ -141,13 +141,25 @@
   </si>
   <si>
     <t>main flow coefficient</t>
+  </si>
+  <si>
+    <t>co-product 6</t>
+  </si>
+  <si>
+    <t>coefficient 6</t>
+  </si>
+  <si>
+    <t>co-product 7</t>
+  </si>
+  <si>
+    <t>coefficient 7</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -202,8 +214,50 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0563C1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF1F497D"/>
+      <name val="Verdana"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -216,8 +270,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDBE5F1"/>
+        <bgColor rgb="FFE4DFEC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor rgb="FFFF9900"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -249,14 +315,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF333F50"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF333F50"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF333F50"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF333F50"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -282,12 +371,23 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="13" fillId="4" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="12">
+    <cellStyle name="Hyperlink 2" xfId="5" xr:uid="{41B8BE02-DEE2-4EB8-9520-5241FB395D5C}"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{2EA035B1-DD36-4732-A763-CAA7E58B5536}"/>
+    <cellStyle name="Normal 2 2" xfId="6" xr:uid="{491B9E03-C7E0-433A-9F99-14719A43CEBE}"/>
+    <cellStyle name="SAPMemberCell" xfId="7" xr:uid="{3A31B2EC-1058-4451-87B6-52EB036C1902}"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2" xfId="2" xr:uid="{B1A8EBD6-8491-4565-9080-220F019946F9}"/>
     <cellStyle name="Standard 2 2" xfId="3" xr:uid="{F92A6CEB-D28B-4DE8-8F32-EE1E95E42DA1}"/>
+    <cellStyle name="Standard 2 2 2" xfId="9" xr:uid="{D8393E1F-A3B1-403D-A27F-3FF577C7E5B7}"/>
+    <cellStyle name="Standard 2 3" xfId="8" xr:uid="{35016BAF-2F51-4BD7-B680-278885866FC9}"/>
+    <cellStyle name="Standard 3" xfId="10" xr:uid="{AFC8C7F1-0088-4313-AE48-8E1013C8BEFC}"/>
+    <cellStyle name="Standard 4" xfId="11" xr:uid="{42E7E662-8B94-4834-AB00-C81213AE3B82}"/>
+    <cellStyle name="Standard 5" xfId="4" xr:uid="{FE6A475C-768A-41A8-B2F1-D0DD66E4EF87}"/>
   </cellStyles>
   <dxfs count="50">
     <dxf>
@@ -1123,7 +1223,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE059C9D-BD0C-48DE-A1E5-C8EAE61483F6}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
   </cols>
@@ -1148,13 +1248,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF9D3058-3D96-495C-ADE7-CBA46DA5595A}">
   <dimension ref="A1:J105"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="32.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="88.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.28515625" customWidth="1"/>
-    <col min="4" max="4" width="16.42578125" customWidth="1"/>
-    <col min="5" max="5" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="32.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="88.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.33203125" customWidth="1"/>
+    <col min="4" max="4" width="16.44140625" customWidth="1"/>
+    <col min="5" max="5" width="18.6640625" customWidth="1"/>
     <col min="8" max="8" width="30" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1563,10 +1663,10 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AE8CFDA-6947-462F-B539-30393EC61A49}">
   <dimension ref="A1:C49"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="69.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="88.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="69.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="88.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1669,18 +1769,18 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2439461A-E0B7-4CD0-B21A-C2DC025CFE6A}">
-  <dimension ref="A1:V52"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="15"/>
+  <dimension ref="A1:Z52"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="88.140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.28515625" customWidth="1"/>
-    <col min="3" max="3" width="39.28515625" style="7" customWidth="1"/>
-    <col min="5" max="5" width="25.28515625" style="7" customWidth="1"/>
-    <col min="7" max="7" width="18.42578125" customWidth="1"/>
-    <col min="13" max="13" width="25.28515625" customWidth="1"/>
+    <col min="1" max="1" width="88.109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.33203125" customWidth="1"/>
+    <col min="3" max="3" width="39.33203125" style="7" customWidth="1"/>
+    <col min="5" max="5" width="25.33203125" style="7" customWidth="1"/>
+    <col min="7" max="7" width="18.44140625" customWidth="1"/>
+    <col min="13" max="13" width="25.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="6" customFormat="1" ht="26.65" customHeight="1">
+    <row r="1" spans="1:26" s="6" customFormat="1" ht="26.7" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>13</v>
       </c>
@@ -1747,78 +1847,90 @@
       <c r="V1" s="3" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:22">
+      <c r="W1" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="X1" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y1" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z1" s="13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26">
       <c r="A2"/>
       <c r="C2"/>
       <c r="E2"/>
     </row>
-    <row r="3" spans="1:22">
+    <row r="3" spans="1:26">
       <c r="A3"/>
       <c r="C3"/>
       <c r="E3"/>
     </row>
-    <row r="4" spans="1:22">
+    <row r="4" spans="1:26">
       <c r="A4"/>
       <c r="C4"/>
       <c r="E4"/>
     </row>
-    <row r="5" spans="1:22">
+    <row r="5" spans="1:26">
       <c r="A5"/>
       <c r="C5"/>
       <c r="E5"/>
     </row>
-    <row r="6" spans="1:22">
+    <row r="6" spans="1:26">
       <c r="A6"/>
       <c r="C6"/>
       <c r="E6"/>
     </row>
-    <row r="7" spans="1:22">
+    <row r="7" spans="1:26">
       <c r="A7"/>
       <c r="C7"/>
       <c r="E7"/>
     </row>
-    <row r="8" spans="1:22">
+    <row r="8" spans="1:26">
       <c r="A8"/>
       <c r="C8"/>
       <c r="E8"/>
     </row>
-    <row r="9" spans="1:22">
+    <row r="9" spans="1:26">
       <c r="A9"/>
       <c r="C9"/>
       <c r="E9"/>
     </row>
-    <row r="10" spans="1:22">
+    <row r="10" spans="1:26">
       <c r="A10"/>
       <c r="C10"/>
       <c r="E10"/>
     </row>
-    <row r="11" spans="1:22">
+    <row r="11" spans="1:26">
       <c r="A11"/>
       <c r="C11"/>
       <c r="E11"/>
     </row>
-    <row r="12" spans="1:22">
+    <row r="12" spans="1:26">
       <c r="A12"/>
       <c r="C12"/>
       <c r="E12"/>
     </row>
-    <row r="13" spans="1:22">
+    <row r="13" spans="1:26">
       <c r="A13"/>
       <c r="C13"/>
       <c r="E13"/>
     </row>
-    <row r="14" spans="1:22">
+    <row r="14" spans="1:26">
       <c r="A14"/>
       <c r="C14"/>
       <c r="E14"/>
     </row>
-    <row r="15" spans="1:22">
+    <row r="15" spans="1:26">
       <c r="A15"/>
       <c r="C15"/>
       <c r="E15"/>
     </row>
-    <row r="16" spans="1:22">
+    <row r="16" spans="1:26">
       <c r="A16"/>
       <c r="C16"/>
       <c r="E16"/>
@@ -1862,10 +1974,10 @@
     <row r="38" spans="1:5">
       <c r="E38"/>
     </row>
-    <row r="39" spans="1:5" ht="18.95" customHeight="1">
+    <row r="39" spans="1:5" ht="18.899999999999999" customHeight="1">
       <c r="C39"/>
     </row>
-    <row r="40" spans="1:5" ht="17.45" customHeight="1">
+    <row r="40" spans="1:5" ht="17.399999999999999" customHeight="1">
       <c r="E40"/>
     </row>
     <row r="41" spans="1:5">
@@ -1930,13 +2042,33 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21588133-5457-4643-8DD0-EFC91AC94F92}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c97a0b29-e816-4eaa-bfb7-7e3a5f017d3a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="865df70f-c489-47a1-8944-6dcc34abd3b0" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100F77CF17864C0D348AA6E64CCBF706952" ma:contentTypeVersion="16" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="c71c6f1ee8c3788f8486deb9f23c45ff">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="865df70f-c489-47a1-8944-6dcc34abd3b0" xmlns:ns3="c97a0b29-e816-4eaa-bfb7-7e3a5f017d3a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ed951fbd2784f2a8953390bad3a39e7a" ns2:_="" ns3:_="">
     <xsd:import namespace="865df70f-c489-47a1-8944-6dcc34abd3b0"/>
@@ -2179,27 +2311,34 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B4F0BBB-F993-4385-BCC0-7127348E19EE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="e2d08c90-bd96-4090-a5fb-15fd3b50eea8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="193a0480-a625-4646-b22e-cb549273dbd4"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="c97a0b29-e816-4eaa-bfb7-7e3a5f017d3a"/>
+    <ds:schemaRef ds:uri="865df70f-c489-47a1-8944-6dcc34abd3b0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c97a0b29-e816-4eaa-bfb7-7e3a5f017d3a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="865df70f-c489-47a1-8944-6dcc34abd3b0" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55565BE3-9439-462C-A1BC-BBE7461E2767}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FAAA6AC-4710-478A-A271-C610929E9C0C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2216,31 +2355,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55565BE3-9439-462C-A1BC-BBE7461E2767}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B4F0BBB-F993-4385-BCC0-7127348E19EE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="e2d08c90-bd96-4090-a5fb-15fd3b50eea8"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="193a0480-a625-4646-b22e-cb549273dbd4"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="c97a0b29-e816-4eaa-bfb7-7e3a5f017d3a"/>
-    <ds:schemaRef ds:uri="865df70f-c489-47a1-8944-6dcc34abd3b0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
change raw material coefficient to rcoefficient in template
</commit_message>
<xml_diff>
--- a/01_create_system_expansion/templates/reaction_extension_layer.xlsx
+++ b/01_create_system_expansion/templates/reaction_extension_layer.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26501"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\gossen\Projects\DB_Improvement\DatabaseGeneration-02_techModel\01_create_system_expansion\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ludwig\Masterthesis\DatabaseGeneration-02_techModel\01_create_system_expansion\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D40AC47E-E838-45DC-B860-DA024CF25A91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30FB0A78-08D8-4B95-9342-BFF87F72CECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-4965" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-3645" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="matrix_table" sheetId="9" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="42">
   <si>
     <t>raw_material_id</t>
   </si>
@@ -153,13 +153,28 @@
   </si>
   <si>
     <t>coefficient 7</t>
+  </si>
+  <si>
+    <t>rcoefficient 1</t>
+  </si>
+  <si>
+    <t>rcoefficient 2</t>
+  </si>
+  <si>
+    <t>rcoefficient 3</t>
+  </si>
+  <si>
+    <t>rcoefficient 4</t>
+  </si>
+  <si>
+    <t>rcoefficient 5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1223,12 +1238,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE059C9D-BD0C-48DE-A1E5-C8EAE61483F6}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -1248,7 +1263,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF9D3058-3D96-495C-ADE7-CBA46DA5595A}">
   <dimension ref="A1:J105"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="88.109375" bestFit="1" customWidth="1"/>
@@ -1258,7 +1273,7 @@
     <col min="8" max="8" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1290,7 +1305,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="1" customFormat="1">
+    <row r="2" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -1307,7 +1322,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:10" s="1" customFormat="1">
+    <row r="3" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -1325,313 +1340,313 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="C17" s="9"/>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
     </row>
-    <row r="30" spans="1:3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
     </row>
-    <row r="31" spans="1:3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
     </row>
-    <row r="33" spans="1:1">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
     </row>
-    <row r="34" spans="1:1">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
     </row>
-    <row r="35" spans="1:1">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
     </row>
-    <row r="36" spans="1:1">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
     </row>
-    <row r="37" spans="1:1">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
     </row>
-    <row r="38" spans="1:1">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
     </row>
-    <row r="39" spans="1:1">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
     </row>
-    <row r="40" spans="1:1">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
     </row>
-    <row r="41" spans="1:1">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
     </row>
-    <row r="42" spans="1:1">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
     </row>
-    <row r="43" spans="1:1">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
     </row>
-    <row r="44" spans="1:1">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
     </row>
-    <row r="45" spans="1:1">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
     </row>
-    <row r="46" spans="1:1">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
     </row>
-    <row r="47" spans="1:1">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
     </row>
-    <row r="48" spans="1:1">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
       <c r="E51" s="11"/>
     </row>
-    <row r="52" spans="1:5">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
     </row>
-    <row r="56" spans="1:5">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
     </row>
-    <row r="57" spans="1:5">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
     </row>
-    <row r="60" spans="1:5">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
     </row>
-    <row r="63" spans="1:5">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
     </row>
-    <row r="64" spans="1:5">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="1"/>
     </row>
-    <row r="65" spans="1:1">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A65" s="1"/>
     </row>
-    <row r="66" spans="1:1">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A66" s="1"/>
     </row>
-    <row r="67" spans="1:1">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
     </row>
-    <row r="68" spans="1:1">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
     </row>
-    <row r="69" spans="1:1">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
     </row>
-    <row r="70" spans="1:1">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A70" s="1"/>
     </row>
-    <row r="71" spans="1:1">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A71" s="1"/>
     </row>
-    <row r="72" spans="1:1">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A72" s="1"/>
     </row>
-    <row r="73" spans="1:1">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A73" s="1"/>
     </row>
-    <row r="74" spans="1:1">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A74" s="1"/>
     </row>
-    <row r="75" spans="1:1">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A75" s="1"/>
     </row>
-    <row r="76" spans="1:1">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A76" s="1"/>
     </row>
-    <row r="77" spans="1:1">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A77" s="1"/>
     </row>
-    <row r="78" spans="1:1">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A78" s="1"/>
     </row>
-    <row r="79" spans="1:1">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A79" s="1"/>
     </row>
-    <row r="80" spans="1:1">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A80" s="1"/>
     </row>
-    <row r="81" spans="1:1">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A81" s="1"/>
     </row>
-    <row r="82" spans="1:1">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A82" s="1"/>
     </row>
-    <row r="83" spans="1:1">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A83" s="1"/>
     </row>
-    <row r="84" spans="1:1">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A84" s="1"/>
     </row>
-    <row r="85" spans="1:1">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A85" s="1"/>
     </row>
-    <row r="86" spans="1:1">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A86" s="1"/>
     </row>
-    <row r="87" spans="1:1">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A87" s="1"/>
     </row>
-    <row r="88" spans="1:1">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A88" s="1"/>
     </row>
-    <row r="89" spans="1:1">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A89" s="1"/>
     </row>
-    <row r="90" spans="1:1">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A90" s="1"/>
     </row>
-    <row r="91" spans="1:1">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A91" s="1"/>
     </row>
-    <row r="92" spans="1:1">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A92" s="1"/>
     </row>
-    <row r="93" spans="1:1">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A93" s="1"/>
     </row>
-    <row r="94" spans="1:1">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A94" s="1"/>
     </row>
-    <row r="95" spans="1:1">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A95" s="1"/>
     </row>
-    <row r="96" spans="1:1">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A96" s="1"/>
     </row>
-    <row r="97" spans="1:3">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A97" s="1"/>
     </row>
-    <row r="98" spans="1:3">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A98" s="1"/>
     </row>
-    <row r="99" spans="1:3">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A99" s="1"/>
     </row>
-    <row r="100" spans="1:3">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A100" s="1"/>
       <c r="C100" s="9"/>
     </row>
-    <row r="101" spans="1:3">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A101" s="1"/>
     </row>
-    <row r="102" spans="1:3">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A102" s="1"/>
     </row>
-    <row r="103" spans="1:3">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A103" s="1"/>
     </row>
-    <row r="104" spans="1:3">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A104" s="1"/>
     </row>
-    <row r="105" spans="1:3">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A105" s="1"/>
     </row>
   </sheetData>
@@ -1663,13 +1678,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AE8CFDA-6947-462F-B539-30393EC61A49}">
   <dimension ref="A1:C49"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="69.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="88.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>29</v>
       </c>
@@ -1680,18 +1695,18 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="3:3">
+    <row r="45" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C45" s="7"/>
     </row>
-    <row r="46" spans="3:3">
+    <row r="46" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C46" s="8"/>
     </row>
-    <row r="49" spans="3:3">
+    <row r="49" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C49" s="10"/>
     </row>
   </sheetData>
@@ -1770,7 +1785,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2439461A-E0B7-4CD0-B21A-C2DC025CFE6A}">
   <dimension ref="A1:Z52"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="88.109375" style="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.33203125" customWidth="1"/>
@@ -1780,7 +1795,7 @@
     <col min="13" max="13" width="25.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" s="6" customFormat="1" ht="26.7" customHeight="1">
+    <row r="1" spans="1:26" s="6" customFormat="1" ht="26.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>13</v>
       </c>
@@ -1791,31 +1806,31 @@
         <v>14</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>16</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>18</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="K1" s="3" t="s">
         <v>22</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="M1" s="5" t="s">
         <v>24</v>
@@ -1860,134 +1875,134 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:26">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A2"/>
       <c r="C2"/>
       <c r="E2"/>
     </row>
-    <row r="3" spans="1:26">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A3"/>
       <c r="C3"/>
       <c r="E3"/>
     </row>
-    <row r="4" spans="1:26">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A4"/>
       <c r="C4"/>
       <c r="E4"/>
     </row>
-    <row r="5" spans="1:26">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A5"/>
       <c r="C5"/>
       <c r="E5"/>
     </row>
-    <row r="6" spans="1:26">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A6"/>
       <c r="C6"/>
       <c r="E6"/>
     </row>
-    <row r="7" spans="1:26">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A7"/>
       <c r="C7"/>
       <c r="E7"/>
     </row>
-    <row r="8" spans="1:26">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A8"/>
       <c r="C8"/>
       <c r="E8"/>
     </row>
-    <row r="9" spans="1:26">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A9"/>
       <c r="C9"/>
       <c r="E9"/>
     </row>
-    <row r="10" spans="1:26">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A10"/>
       <c r="C10"/>
       <c r="E10"/>
     </row>
-    <row r="11" spans="1:26">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A11"/>
       <c r="C11"/>
       <c r="E11"/>
     </row>
-    <row r="12" spans="1:26">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A12"/>
       <c r="C12"/>
       <c r="E12"/>
     </row>
-    <row r="13" spans="1:26">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A13"/>
       <c r="C13"/>
       <c r="E13"/>
     </row>
-    <row r="14" spans="1:26">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A14"/>
       <c r="C14"/>
       <c r="E14"/>
     </row>
-    <row r="15" spans="1:26">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A15"/>
       <c r="C15"/>
       <c r="E15"/>
     </row>
-    <row r="16" spans="1:26">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A16"/>
       <c r="C16"/>
       <c r="E16"/>
     </row>
-    <row r="17" customFormat="1"/>
-    <row r="18" customFormat="1"/>
-    <row r="19" customFormat="1"/>
-    <row r="20" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="21" customFormat="1"/>
-    <row r="22" customFormat="1"/>
-    <row r="23" customFormat="1"/>
-    <row r="24" customFormat="1"/>
-    <row r="25" customFormat="1"/>
-    <row r="26" customFormat="1"/>
-    <row r="27" customFormat="1"/>
-    <row r="28" customFormat="1"/>
-    <row r="29" customFormat="1"/>
-    <row r="30" customFormat="1"/>
-    <row r="31" customFormat="1"/>
-    <row r="32" customFormat="1"/>
-    <row r="33" spans="1:5">
+    <row r="17" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="18" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="19" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="20" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="21" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="22" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="23" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="24" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="25" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="26" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="27" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="28" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="29" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="30" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="31" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="32" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33"/>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C34"/>
       <c r="E34"/>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35"/>
       <c r="E35"/>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36"/>
       <c r="C36"/>
       <c r="E36"/>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37"/>
       <c r="E37"/>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E38"/>
     </row>
-    <row r="39" spans="1:5" ht="18.899999999999999" customHeight="1">
+    <row r="39" spans="1:5" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C39"/>
     </row>
-    <row r="40" spans="1:5" ht="17.399999999999999" customHeight="1">
+    <row r="40" spans="1:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E40"/>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E41"/>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C42"/>
       <c r="E42"/>
     </row>
-    <row r="52" ht="16.5" customHeight="1"/>
+    <row r="52" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <conditionalFormatting sqref="A2:A44">
     <cfRule type="duplicateValues" dxfId="15" priority="510"/>
@@ -2042,33 +2057,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21588133-5457-4643-8DD0-EFC91AC94F92}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c97a0b29-e816-4eaa-bfb7-7e3a5f017d3a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="865df70f-c489-47a1-8944-6dcc34abd3b0" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100F77CF17864C0D348AA6E64CCBF706952" ma:contentTypeVersion="16" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="c71c6f1ee8c3788f8486deb9f23c45ff">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="865df70f-c489-47a1-8944-6dcc34abd3b0" xmlns:ns3="c97a0b29-e816-4eaa-bfb7-7e3a5f017d3a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ed951fbd2784f2a8953390bad3a39e7a" ns2:_="" ns3:_="">
     <xsd:import namespace="865df70f-c489-47a1-8944-6dcc34abd3b0"/>
@@ -2311,7 +2306,54 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c97a0b29-e816-4eaa-bfb7-7e3a5f017d3a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="865df70f-c489-47a1-8944-6dcc34abd3b0" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FAAA6AC-4710-478A-A271-C610929E9C0C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="865df70f-c489-47a1-8944-6dcc34abd3b0"/>
+    <ds:schemaRef ds:uri="c97a0b29-e816-4eaa-bfb7-7e3a5f017d3a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55565BE3-9439-462C-A1BC-BBE7461E2767}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B4F0BBB-F993-4385-BCC0-7127348E19EE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
@@ -2328,31 +2370,4 @@
     <ds:schemaRef ds:uri="865df70f-c489-47a1-8944-6dcc34abd3b0"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55565BE3-9439-462C-A1BC-BBE7461E2767}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FAAA6AC-4710-478A-A271-C610929E9C0C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="865df70f-c489-47a1-8944-6dcc34abd3b0"/>
-    <ds:schemaRef ds:uri="c97a0b29-e816-4eaa-bfb7-7e3a5f017d3a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>